<commit_message>
fix(seeding): update service ID lookup to use service name instead of code
</commit_message>
<xml_diff>
--- a/data/Data Membership.xlsx
+++ b/data/Data Membership.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="41">
   <si>
     <t>name</t>
   </si>
@@ -91,13 +91,16 @@
     <t xml:space="preserve">VIP - Home 6 Months </t>
   </si>
   <si>
+    <t xml:space="preserve">Basic Grooming - Home Service </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full Grooming - Home Service </t>
+  </si>
+  <si>
     <t xml:space="preserve">VIP - In Store 12 Months </t>
   </si>
   <si>
-    <t xml:space="preserve">Basic Grooming - Home Service </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full Grooming - Home Service </t>
+    <t xml:space="preserve">Basic Grooming - In Store </t>
   </si>
   <si>
     <t xml:space="preserve">VIP - Home 12 Months </t>
@@ -244,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -280,7 +283,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="6" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -509,7 +518,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="22.88"/>
     <col customWidth="1" min="3" max="3" width="17.13"/>
-    <col customWidth="1" min="9" max="9" width="24.25"/>
+    <col customWidth="1" min="9" max="9" width="28.5"/>
     <col customWidth="1" min="10" max="10" width="20.5"/>
   </cols>
   <sheetData>
@@ -680,18 +689,18 @@
       <c r="H6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="J6" s="14"/>
+      <c r="I6" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="15"/>
       <c r="K6" s="6" t="s">
         <v>19</v>
       </c>
       <c r="L6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="M6" s="14"/>
-      <c r="N6" s="14"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="15"/>
     </row>
     <row r="7">
       <c r="A7" s="11"/>
@@ -704,18 +713,18 @@
       <c r="H7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="J7" s="14"/>
+      <c r="I7" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="15"/>
       <c r="K7" s="6" t="s">
         <v>19</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="M7" s="14"/>
-      <c r="N7" s="14"/>
+      <c r="M7" s="15"/>
+      <c r="N7" s="15"/>
     </row>
     <row r="8">
       <c r="A8" s="5"/>
@@ -728,7 +737,7 @@
       <c r="H8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="I8" s="14"/>
+      <c r="I8" s="15"/>
       <c r="J8" s="6" t="s">
         <v>23</v>
       </c>
@@ -738,14 +747,14 @@
       <c r="L8" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="M8" s="14"/>
+      <c r="M8" s="15"/>
       <c r="N8" s="6">
         <v>10.0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="8">
@@ -764,8 +773,8 @@
       <c r="H9" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="9" t="s">
-        <v>27</v>
+      <c r="I9" s="16" t="s">
+        <v>29</v>
       </c>
       <c r="J9" s="10"/>
       <c r="K9" s="9" t="s">
@@ -788,8 +797,8 @@
       <c r="H10" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="9" t="s">
-        <v>28</v>
+      <c r="I10" s="16" t="s">
+        <v>21</v>
       </c>
       <c r="J10" s="10"/>
       <c r="K10" s="9" t="s">
@@ -829,7 +838,7 @@
     </row>
     <row r="12">
       <c r="A12" s="12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="13">
@@ -849,17 +858,17 @@
         <v>17</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="J12" s="14"/>
+        <v>26</v>
+      </c>
+      <c r="J12" s="15"/>
       <c r="K12" s="6" t="s">
         <v>19</v>
       </c>
       <c r="L12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="M12" s="14"/>
-      <c r="N12" s="14"/>
+      <c r="M12" s="15"/>
+      <c r="N12" s="15"/>
     </row>
     <row r="13">
       <c r="A13" s="11"/>
@@ -873,17 +882,17 @@
         <v>17</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="J13" s="14"/>
+        <v>27</v>
+      </c>
+      <c r="J13" s="15"/>
       <c r="K13" s="6" t="s">
         <v>19</v>
       </c>
       <c r="L13" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="M13" s="14"/>
-      <c r="N13" s="14"/>
+      <c r="M13" s="15"/>
+      <c r="N13" s="15"/>
     </row>
     <row r="14">
       <c r="A14" s="5"/>
@@ -896,7 +905,7 @@
       <c r="H14" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="I14" s="14"/>
+      <c r="I14" s="15"/>
       <c r="J14" s="6" t="s">
         <v>23</v>
       </c>
@@ -906,14 +915,14 @@
       <c r="L14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="M14" s="14"/>
+      <c r="M14" s="15"/>
       <c r="N14" s="6">
         <v>10.0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="8">
@@ -929,23 +938,23 @@
       <c r="G15" s="8" t="b">
         <v>1</v>
       </c>
-      <c r="H15" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="I15" s="15" t="s">
+      <c r="H15" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="I15" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="J15" s="16"/>
-      <c r="K15" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="L15" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="M15" s="15">
+      <c r="J15" s="18"/>
+      <c r="K15" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="L15" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="M15" s="17">
         <v>1.0</v>
       </c>
-      <c r="N15" s="16"/>
+      <c r="N15" s="18"/>
     </row>
     <row r="16">
       <c r="A16" s="11"/>
@@ -955,23 +964,23 @@
       <c r="E16" s="11"/>
       <c r="F16" s="11"/>
       <c r="G16" s="11"/>
-      <c r="H16" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="I16" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="J16" s="16"/>
-      <c r="K16" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="L16" s="15" t="s">
+      <c r="H16" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="I16" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="M16" s="15">
+      <c r="J16" s="18"/>
+      <c r="K16" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="L16" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="M16" s="17">
         <v>1.0</v>
       </c>
-      <c r="N16" s="16"/>
+      <c r="N16" s="18"/>
     </row>
     <row r="17">
       <c r="A17" s="5"/>
@@ -981,29 +990,29 @@
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
-      <c r="H17" s="15" t="s">
+      <c r="H17" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I17" s="16"/>
-      <c r="J17" s="15" t="s">
+      <c r="I17" s="18"/>
+      <c r="J17" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="K17" s="15" t="s">
+      <c r="K17" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="L17" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="M17" s="15">
+      <c r="L17" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="M17" s="17">
         <v>1.0</v>
       </c>
-      <c r="N17" s="15">
+      <c r="N17" s="17">
         <v>10.0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="13">
@@ -1019,23 +1028,23 @@
       <c r="G18" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="H18" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="I18" s="17" t="s">
+      <c r="H18" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="I18" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="J18" s="18"/>
-      <c r="K18" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="L18" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="M18" s="17">
+      <c r="J18" s="20"/>
+      <c r="K18" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="L18" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="M18" s="19">
         <v>1.0</v>
       </c>
-      <c r="N18" s="18"/>
+      <c r="N18" s="20"/>
     </row>
     <row r="19">
       <c r="A19" s="11"/>
@@ -1045,23 +1054,23 @@
       <c r="E19" s="11"/>
       <c r="F19" s="11"/>
       <c r="G19" s="11"/>
-      <c r="H19" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="I19" s="17" t="s">
+      <c r="H19" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="I19" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="J19" s="18"/>
-      <c r="K19" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="L19" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="M19" s="17">
+      <c r="J19" s="20"/>
+      <c r="K19" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="L19" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="M19" s="19">
         <v>1.0</v>
       </c>
-      <c r="N19" s="18"/>
+      <c r="N19" s="20"/>
     </row>
     <row r="20">
       <c r="A20" s="11"/>
@@ -1071,23 +1080,23 @@
       <c r="E20" s="11"/>
       <c r="F20" s="11"/>
       <c r="G20" s="11"/>
-      <c r="H20" s="17" t="s">
+      <c r="H20" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="I20" s="18"/>
-      <c r="J20" s="17" t="s">
+      <c r="I20" s="20"/>
+      <c r="J20" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="K20" s="17" t="s">
+      <c r="K20" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="L20" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="M20" s="17">
+      <c r="L20" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="M20" s="19">
         <v>1.0</v>
       </c>
-      <c r="N20" s="17">
+      <c r="N20" s="19">
         <v>10.0</v>
       </c>
     </row>
@@ -1099,27 +1108,27 @@
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
-      <c r="H21" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I21" s="18"/>
-      <c r="J21" s="17" t="s">
+      <c r="H21" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="K21" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="L21" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="M21" s="17">
+      <c r="I21" s="20"/>
+      <c r="J21" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="K21" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="L21" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="M21" s="19">
         <v>1.0</v>
       </c>
-      <c r="N21" s="18"/>
+      <c r="N21" s="20"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="8">
@@ -1135,23 +1144,23 @@
       <c r="G22" s="8" t="b">
         <v>1</v>
       </c>
-      <c r="H22" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="I22" s="15" t="s">
+      <c r="H22" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="J22" s="16"/>
-      <c r="K22" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="L22" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="M22" s="15">
+      <c r="J22" s="18"/>
+      <c r="K22" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="L22" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="M22" s="17">
         <v>1.0</v>
       </c>
-      <c r="N22" s="16"/>
+      <c r="N22" s="18"/>
     </row>
     <row r="23">
       <c r="A23" s="11"/>
@@ -1161,23 +1170,23 @@
       <c r="E23" s="11"/>
       <c r="F23" s="11"/>
       <c r="G23" s="11"/>
-      <c r="H23" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="I23" s="15" t="s">
+      <c r="H23" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="I23" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="J23" s="16"/>
-      <c r="K23" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="L23" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="M23" s="15">
+      <c r="J23" s="18"/>
+      <c r="K23" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="L23" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="M23" s="17">
         <v>1.0</v>
       </c>
-      <c r="N23" s="16"/>
+      <c r="N23" s="18"/>
     </row>
     <row r="24">
       <c r="A24" s="11"/>
@@ -1187,23 +1196,23 @@
       <c r="E24" s="11"/>
       <c r="F24" s="11"/>
       <c r="G24" s="11"/>
-      <c r="H24" s="15" t="s">
+      <c r="H24" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="16"/>
-      <c r="J24" s="15" t="s">
+      <c r="I24" s="18"/>
+      <c r="J24" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="K24" s="15" t="s">
+      <c r="K24" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="L24" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="M24" s="15">
+      <c r="L24" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="M24" s="17">
         <v>1.0</v>
       </c>
-      <c r="N24" s="15">
+      <c r="N24" s="17">
         <v>10.0</v>
       </c>
     </row>
@@ -1215,21 +1224,21 @@
       <c r="E25" s="11"/>
       <c r="F25" s="11"/>
       <c r="G25" s="11"/>
-      <c r="H25" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="I25" s="16"/>
-      <c r="J25" s="15" t="s">
+      <c r="H25" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="K25" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="L25" s="15" t="s">
+      <c r="I25" s="18"/>
+      <c r="J25" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="K25" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="L25" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="M25" s="16"/>
-      <c r="N25" s="16"/>
+      <c r="M25" s="18"/>
+      <c r="N25" s="18"/>
     </row>
     <row r="26">
       <c r="A26" s="11"/>
@@ -1239,23 +1248,23 @@
       <c r="E26" s="11"/>
       <c r="F26" s="11"/>
       <c r="G26" s="11"/>
-      <c r="H26" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="I26" s="16"/>
-      <c r="J26" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="K26" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="L26" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="M26" s="15">
+      <c r="H26" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="I26" s="18"/>
+      <c r="J26" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="K26" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="L26" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="M26" s="17">
         <v>4.0</v>
       </c>
-      <c r="N26" s="16"/>
+      <c r="N26" s="18"/>
     </row>
     <row r="27">
       <c r="A27" s="5"/>
@@ -1265,23 +1274,23 @@
       <c r="E27" s="5"/>
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
-      <c r="H27" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="I27" s="16"/>
-      <c r="J27" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="K27" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="L27" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="M27" s="15">
+      <c r="H27" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="I27" s="18"/>
+      <c r="J27" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="K27" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="L27" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="M27" s="17">
         <v>1.0</v>
       </c>
-      <c r="N27" s="16"/>
+      <c r="N27" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="57">

</xml_diff>